<commit_message>
feat(cli): dsl parse/check/generate/build 命令行工具（dev/22）
- packages/cli（bin dsl）：多文件目录入口（顶层 *.tdsl 排序）→ parseProject（M7）
- 薄命令层：run(argv)→{code,stdout} 结构化结果，可测可复用（编译服务地基）
- app 名：--name 或目录名清洗为合法 Java 标识符（codegen 校验为最后防线）
- 诊断人话化：[severity] file path: message；<stdin> 隐藏
- 零新增依赖：argv 手写解析；bin 经 tsx ESM register 加载 TS 源（不开构建链）
- 验收：dsl build examples/todo-multi/tdsl 双端 build 通过；坏分片 → exit 1
- 测试: 155 → 169（cli +14）；根 package.json 接入 npm run dsl + 八包 typecheck
- 踩坑入库: type AppNode 从 parser 导入但未导出 → TS 静默 any，语义核类型一律从 core 导入
</commit_message>
<xml_diff>
--- a/docs/dev/QA记录.xlsx
+++ b/docs/dev/QA记录.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,156 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>M7 拆分标准：按功能纵向切（用户确认），共享数据模型独立文件，跨文件引用最少；语言层零约束，拆法是使用策略</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>M7 拆分方式：import vs 全局命名空间</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>全局命名空间（对标 NASL，无 import），link 前合并</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>M7 发现既有 bug：declareGlobal 以 existing!==path 判重，同名 logic path 恒等导致同段重名一直漏报</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>收紧为同 path 也报错，新增双文件报错单测</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>M7 app 名带连字符（todo-multi）→ Java 包名/类名非法，此前硬编码 todo 未暴露</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>codegen-java pkgOf 入口校验合法 Java 标识符并抛错；示例改用 todomulti</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>M7 对拍首跑失败：两侧 app 名不同致包名/路径全不同（非语义漂移）</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>app 名是入参非解析产物，对拍前对齐 singleApp.name</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>M8 CLI 运行形态：不开构建链，bin 经 tsx ESM register 加载 TS 源（与全仓 packages main=src/index.ts 形态一致）</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>M8 发现 type AppNode 从 @tdsl/parser 导入但 parser 不导出该类型，TS 静默当 any（隐式 any 报错才暴露）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>语义核类型一律从 @tdsl/core 导入，已入库踩坑</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>M8 build 端到端：dsl build examples/todo-multi/tdsl -o generated → mvn compile + vite build 通过（java 20 + react 12 files）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>已验证</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(m11): dev/49-51 需求/系统/详细设计 + 语法手册鉴权章与 ! 漂移修正 + cheatsheet 同步 + index/QA/memory
</commit_message>
<xml_diff>
--- a/docs/dev/QA记录.xlsx
+++ b/docs/dev/QA记录.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1047,6 +1047,106 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>M11 鉴权：FFI_CORE 五域守门测试撞 Auth 域</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>按新口径更新：五语言域 + 平台鉴权域（无 maven 坐标，internal 标记 import 跳过）</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>M11 块注释 /* */ 不被 lexer 支持（yudao 70-auth.tdsl 样例报 unexpected char）</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>确认边界：lexer 仅 //；样例改行注释；块注释支持列为独立余项</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>M11 语言边界：无一元 !（手册漂移）；List.get(0) 字段访问 java 无类型通道</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>样例用 for-of 与 === false 规避；语法手册 §2 漂移已修；get(0) 通道留 M3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>M11 react：公开页 Space 多收致 TS6133 / register 成功链 d 未用 / RequireAuth 包装正则</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>collectAntdComponents 按 @public 排除动作区组件；successChain 按是否用返回值选形；改为构造期包装</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>M11 register 接口返回实体会带出密码哈希</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>演示口径可接受；商用需投影脱敏（记录为余项）</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>保持观察</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>